<commit_message>
Substitui projeto pelo dashboard Saídas BEL
</commit_message>
<xml_diff>
--- a/Saida_BEL.xlsx
+++ b/Saida_BEL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Manoel\Documents\project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Manoel\Documents\saidas_bel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35F9B2DC-5A4F-44D4-B2E9-086BD89E2BF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{579DD06C-AC66-47DE-8C2D-CABEC6707E6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{B4DF3242-8F2B-4ADB-9A16-64AB3DBBB1AB}"/>
   </bookViews>
@@ -13351,19 +13351,19 @@
         <v>13</v>
       </c>
       <c r="S126" s="4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="T126" s="12">
         <f>Tabela32[[#This Row],[Entregas]]-Tabela32[[#This Row],[Realizadas]]</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U126" s="18">
         <f>Tabela32[[#This Row],[Realizadas]]/Tabela32[[#This Row],[Entregas]]</f>
-        <v>1</v>
+        <v>0.84615384615384615</v>
       </c>
       <c r="V126" s="19" t="str">
         <f>IF(Tabela32[[#This Row],[% Entrega]]&gt;=96%,"Atendeu a Meta","Não Atendeu a Meta")</f>
-        <v>Atendeu a Meta</v>
+        <v>Não Atendeu a Meta</v>
       </c>
       <c r="W126" s="4" t="s">
         <v>40</v>

</xml_diff>